<commit_message>
migrating content template pages, header, footer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 79
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-landing-page.report.xlsx
+++ b/tools/importer/reports/import-content-landing-page.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="107">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,24 @@
     <t>url</t>
   </si>
   <si>
+    <t>footer.report.json</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>footer</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>2026-10-05T18:08:40.243Z</t>
+  </si>
+  <si>
+    <t>https://www.destinationpet.com/</t>
+  </si>
+  <si>
     <t>index.report.json</t>
   </si>
   <si>
@@ -46,21 +64,15 @@
     <t>index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>content-landing-page</t>
   </si>
   <si>
-    <t>2026-10-05T13:45:07.471Z</t>
+    <t>2026-10-06T07:03:54.141Z</t>
   </si>
   <si>
     <t>Home - Pet Care Network | Destination Pet</t>
   </si>
   <si>
-    <t>https://www.destinationpet.com/</t>
-  </si>
-  <si>
     <t>live-webinar.report.json</t>
   </si>
   <si>
@@ -70,7 +82,7 @@
     <t>live-webinar</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:19.316Z</t>
+    <t>2026-10-06T07:04:37.067Z</t>
   </si>
   <si>
     <t>A Series of Webinars | Destination Pet</t>
@@ -79,6 +91,15 @@
     <t>https://www.destinationpet.com/live-webinar/</t>
   </si>
   <si>
+    <t>nav.report.json</t>
+  </si>
+  <si>
+    <t>nav</t>
+  </si>
+  <si>
+    <t>2026-10-05T17:23:53.482Z</t>
+  </si>
+  <si>
     <t>our-locations.report.json</t>
   </si>
   <si>
@@ -88,7 +109,7 @@
     <t>our-locations</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:47.608Z</t>
+    <t>2026-10-06T07:05:44.949Z</t>
   </si>
   <si>
     <t>Our Locations | Destination Pet</t>
@@ -106,7 +127,7 @@
     <t>sell-your-business</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:53.683Z</t>
+    <t>2026-10-06T07:05:13.807Z</t>
   </si>
   <si>
     <t>Sell Your Veterinary | Destination Pet</t>
@@ -124,7 +145,7 @@
     <t>about-us/about</t>
   </si>
   <si>
-    <t>2026-10-05T13:45:39.341Z</t>
+    <t>2026-10-06T07:03:59.368Z</t>
   </si>
   <si>
     <t>About Us | Destination Pet, LLC</t>
@@ -142,7 +163,7 @@
     <t>about-us/get-in-touch</t>
   </si>
   <si>
-    <t>2026-10-05T13:45:47.855Z</t>
+    <t>2026-10-06T07:04:06.632Z</t>
   </si>
   <si>
     <t>Contact Us | Destination Pet, LLC</t>
@@ -157,7 +178,7 @@
     <t>join-our-pack/find-a-veterinary-externship</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:08.288Z</t>
+    <t>2026-10-06T07:04:26.193Z</t>
   </si>
   <si>
     <t>Find a Veterinary Externship - Destination Pet</t>
@@ -175,7 +196,7 @@
     <t>join-our-pack/life-at-dp</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:12.606Z</t>
+    <t>2026-10-06T07:04:32.565Z</t>
   </si>
   <si>
     <t>life at Destination Pet | Destination Pet</t>
@@ -193,7 +214,7 @@
     <t>live-webinar/webinar-redirect</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:24.311Z</t>
+    <t>2026-10-06T07:04:42.325Z</t>
   </si>
   <si>
     <t>Webinar Redirect - Destination Pet</t>
@@ -208,7 +229,7 @@
     <t>live-webinar/webinar-registration</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:29.670Z</t>
+    <t>2026-10-06T07:04:47.899Z</t>
   </si>
   <si>
     <t>Webinar Registration - Destination Pet</t>
@@ -223,7 +244,7 @@
     <t>live-webinar/webinar-viewing-previous</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:35.996Z</t>
+    <t>2026-10-06T07:04:53.143Z</t>
   </si>
   <si>
     <t>Webinar Viewing Previous - Destination Pet</t>
@@ -238,7 +259,7 @@
     <t>live-webinar/webinars-for-pet</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:41.849Z</t>
+    <t>2026-10-06T07:04:59.003Z</t>
   </si>
   <si>
     <t>Webinars for Pet - Destination Pet</t>
@@ -256,7 +277,7 @@
     <t>sell-your-business/sell-your-pet-resort</t>
   </si>
   <si>
-    <t>2026-10-05T13:47:00.170Z</t>
+    <t>2026-10-06T07:05:18.864Z</t>
   </si>
   <si>
     <t>Sell Your Pet Resort - Destination Pet</t>
@@ -274,7 +295,7 @@
     <t>sell-your-business/sell-your-veterinary-practice</t>
   </si>
   <si>
-    <t>2026-10-05T13:47:05.999Z</t>
+    <t>2026-10-06T07:05:23.774Z</t>
   </si>
   <si>
     <t>Sell your veterinary practice | Destination Pet</t>
@@ -289,7 +310,7 @@
     <t>about-us/meet-the-team/business-development-leaders</t>
   </si>
   <si>
-    <t>2026-10-05T13:45:52.450Z</t>
+    <t>2026-10-06T07:04:12.956Z</t>
   </si>
   <si>
     <t>Business Development Leaders | Destination Pet</t>
@@ -304,7 +325,7 @@
     <t>about-us/meet-the-team/leadership</t>
   </si>
   <si>
-    <t>2026-10-05T13:46:01.550Z</t>
+    <t>2026-10-06T07:04:18.758Z</t>
   </si>
   <si>
     <t>Leadership - Meet the team | Destination Pet</t>
@@ -699,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="3" width="50" customWidth="1"/>
@@ -749,406 +770,458 @@
         <v>11</v>
       </c>
       <c r="E2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" t="s">
         <v>12</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2" t="s">
         <v>13</v>
-      </c>
-      <c r="G2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
-        <v>12</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="G3" t="s">
-        <v>20</v>
-      </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
         <v>23</v>
       </c>
-      <c r="C4" t="s">
+      <c r="G4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" t="s">
+      <c r="H4" t="s">
         <v>25</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>28</v>
       </c>
-      <c r="B5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
-        <v>31</v>
-      </c>
       <c r="G5" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H5" t="s">
-        <v>33</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
         <v>34</v>
-      </c>
-      <c r="B6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="s">
-        <v>37</v>
-      </c>
-      <c r="G6" t="s">
-        <v>38</v>
-      </c>
-      <c r="H6" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" t="s">
         <v>40</v>
-      </c>
-      <c r="B7" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="s">
-        <v>43</v>
-      </c>
-      <c r="G7" t="s">
-        <v>44</v>
-      </c>
-      <c r="H7" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" t="s">
+        <v>45</v>
+      </c>
+      <c r="H8" t="s">
         <v>46</v>
-      </c>
-      <c r="B8" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" t="s">
-        <v>47</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" t="s">
-        <v>49</v>
-      </c>
-      <c r="H8" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" t="s">
+        <v>48</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" t="s">
         <v>51</v>
       </c>
-      <c r="B9" t="s">
+      <c r="H9" t="s">
         <v>52</v>
-      </c>
-      <c r="C9" t="s">
-        <v>53</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="s">
-        <v>54</v>
-      </c>
-      <c r="G9" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" t="s">
+        <v>54</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" t="s">
+        <v>55</v>
+      </c>
+      <c r="G10" t="s">
+        <v>56</v>
+      </c>
+      <c r="H10" t="s">
         <v>57</v>
-      </c>
-      <c r="B10" t="s">
-        <v>58</v>
-      </c>
-      <c r="C10" t="s">
-        <v>59</v>
-      </c>
-      <c r="D10" t="s">
-        <v>11</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="s">
-        <v>60</v>
-      </c>
-      <c r="G10" t="s">
-        <v>61</v>
-      </c>
-      <c r="H10" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>17</v>
+      </c>
+      <c r="F11" t="s">
+        <v>61</v>
+      </c>
+      <c r="G11" t="s">
+        <v>62</v>
+      </c>
+      <c r="H11" t="s">
         <v>63</v>
-      </c>
-      <c r="B11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C11" t="s">
-        <v>64</v>
-      </c>
-      <c r="D11" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" t="s">
-        <v>12</v>
-      </c>
-      <c r="F11" t="s">
-        <v>65</v>
-      </c>
-      <c r="G11" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" t="s">
         <v>68</v>
       </c>
-      <c r="B12" t="s">
-        <v>41</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="H12" t="s">
         <v>69</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>12</v>
-      </c>
-      <c r="F12" t="s">
-        <v>70</v>
-      </c>
-      <c r="G12" t="s">
-        <v>71</v>
-      </c>
-      <c r="H12" t="s">
-        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>70</v>
+      </c>
+      <c r="B13" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" t="s">
         <v>73</v>
       </c>
-      <c r="B13" t="s">
-        <v>58</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="H13" t="s">
         <v>74</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F13" t="s">
-        <v>75</v>
-      </c>
-      <c r="G13" t="s">
-        <v>76</v>
-      </c>
-      <c r="H13" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
+        <v>75</v>
+      </c>
+      <c r="B14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" t="s">
         <v>78</v>
       </c>
-      <c r="B14" t="s">
+      <c r="H14" t="s">
         <v>79</v>
-      </c>
-      <c r="C14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" t="s">
-        <v>11</v>
-      </c>
-      <c r="E14" t="s">
-        <v>12</v>
-      </c>
-      <c r="F14" t="s">
-        <v>81</v>
-      </c>
-      <c r="G14" t="s">
-        <v>82</v>
-      </c>
-      <c r="H14" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>80</v>
+      </c>
+      <c r="B15" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F15" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" t="s">
         <v>84</v>
-      </c>
-      <c r="B15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C15" t="s">
-        <v>86</v>
-      </c>
-      <c r="D15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" t="s">
-        <v>87</v>
-      </c>
-      <c r="G15" t="s">
-        <v>88</v>
-      </c>
-      <c r="H15" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C16" t="s">
+        <v>87</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>17</v>
+      </c>
+      <c r="F16" t="s">
+        <v>88</v>
+      </c>
+      <c r="G16" t="s">
+        <v>89</v>
+      </c>
+      <c r="H16" t="s">
         <v>90</v>
-      </c>
-      <c r="B16" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" t="s">
-        <v>91</v>
-      </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>12</v>
-      </c>
-      <c r="F16" t="s">
-        <v>92</v>
-      </c>
-      <c r="G16" t="s">
-        <v>93</v>
-      </c>
-      <c r="H16" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>91</v>
+      </c>
+      <c r="B17" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" t="s">
+        <v>93</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>17</v>
+      </c>
+      <c r="F17" t="s">
+        <v>94</v>
+      </c>
+      <c r="G17" t="s">
         <v>95</v>
       </c>
-      <c r="B17" t="s">
-        <v>35</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="H17" t="s">
         <v>96</v>
       </c>
-      <c r="D17" t="s">
-        <v>11</v>
-      </c>
-      <c r="E17" t="s">
-        <v>12</v>
-      </c>
-      <c r="F17" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>97</v>
       </c>
-      <c r="G17" t="s">
+      <c r="B18" t="s">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s">
         <v>98</v>
       </c>
-      <c r="H17" t="s">
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>17</v>
+      </c>
+      <c r="F18" t="s">
         <v>99</v>
+      </c>
+      <c r="G18" t="s">
+        <v>100</v>
+      </c>
+      <c r="H18" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B19" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" t="s">
+        <v>104</v>
+      </c>
+      <c r="G19" t="s">
+        <v>105</v>
+      </c>
+      <c r="H19" t="s">
+        <v>106</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
critique AEM authoring in UED
Automated migration updates generated by Experience Modernization Agent.

Changed files: 67
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-content-landing-page.report.xlsx
+++ b/tools/importer/reports/import-content-landing-page.report.xlsx
@@ -103,7 +103,7 @@
     <t>content-landing-page</t>
   </si>
   <si>
-    <t>2026-10-13T14:47:37.751Z</t>
+    <t>2026-10-13T15:19:52.095Z</t>
   </si>
   <si>
     <t>Home - Pet Care Network | Destination Pet</t>
@@ -136,7 +136,7 @@
     <t>live-webinar</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:16.811Z</t>
+    <t>2026-10-13T15:20:32.988Z</t>
   </si>
   <si>
     <t>A Series of Webinars | Destination Pet</t>
@@ -163,7 +163,7 @@
     <t>our-locations</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:43.745Z</t>
+    <t>2026-10-13T15:20:59.607Z</t>
   </si>
   <si>
     <t>Our Locations | Destination Pet</t>
@@ -199,7 +199,7 @@
     <t>sell-your-business</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:49.013Z</t>
+    <t>2026-10-13T15:21:05.928Z</t>
   </si>
   <si>
     <t>Sell Your Veterinary | Destination Pet</t>
@@ -232,7 +232,7 @@
     <t>about-us/about</t>
   </si>
   <si>
-    <t>2026-10-13T14:47:42.734Z</t>
+    <t>2026-10-13T15:19:57.662Z</t>
   </si>
   <si>
     <t>About Us | Destination Pet, LLC</t>
@@ -268,7 +268,7 @@
     <t>hero-feature-showcase</t>
   </si>
   <si>
-    <t>2026-10-13T14:28:37.671Z</t>
+    <t>2026-10-13T14:49:04.899Z</t>
   </si>
   <si>
     <t>Destination Pet Foundation - Destination Pet</t>
@@ -286,7 +286,7 @@
     <t>about-us/get-in-touch</t>
   </si>
   <si>
-    <t>2026-10-13T14:47:49.688Z</t>
+    <t>2026-10-13T15:20:04.813Z</t>
   </si>
   <si>
     <t>Contact Us | Destination Pet, LLC</t>
@@ -334,7 +334,7 @@
     <t>join-our-pack/find-a-veterinary-externship</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:05.794Z</t>
+    <t>2026-10-13T15:20:23.797Z</t>
   </si>
   <si>
     <t>Find a Veterinary Externship - Destination Pet</t>
@@ -352,7 +352,7 @@
     <t>join-our-pack/life-at-dp</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:10.944Z</t>
+    <t>2026-10-13T15:20:27.908Z</t>
   </si>
   <si>
     <t>life at Destination Pet | Destination Pet</t>
@@ -370,7 +370,7 @@
     <t>live-webinar/webinar-redirect</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:22.095Z</t>
+    <t>2026-10-13T15:20:36.986Z</t>
   </si>
   <si>
     <t>Webinar Redirect - Destination Pet</t>
@@ -385,7 +385,7 @@
     <t>live-webinar/webinar-registration</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:26.295Z</t>
+    <t>2026-10-13T15:20:42.646Z</t>
   </si>
   <si>
     <t>Webinar Registration - Destination Pet</t>
@@ -400,7 +400,7 @@
     <t>live-webinar/webinar-viewing-previous</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:32.499Z</t>
+    <t>2026-10-13T15:20:48.822Z</t>
   </si>
   <si>
     <t>Webinar Viewing Previous - Destination Pet</t>
@@ -415,7 +415,7 @@
     <t>live-webinar/webinars-for-pet</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:37.463Z</t>
+    <t>2026-10-13T15:20:53.204Z</t>
   </si>
   <si>
     <t>Webinars for Pet - Destination Pet</t>
@@ -454,7 +454,7 @@
     <t>sell-your-business/sell-your-pet-resort</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:53.416Z</t>
+    <t>2026-10-13T15:21:11.714Z</t>
   </si>
   <si>
     <t>Sell Your Pet Resort - Destination Pet</t>
@@ -472,7 +472,7 @@
     <t>sell-your-business/sell-your-veterinary-practice</t>
   </si>
   <si>
-    <t>2026-10-13T14:48:59.762Z</t>
+    <t>2026-10-13T15:21:16.461Z</t>
   </si>
   <si>
     <t>Sell your veterinary practice | Destination Pet</t>
@@ -487,7 +487,7 @@
     <t>about-us/meet-the-team/business-development-leaders</t>
   </si>
   <si>
-    <t>2026-10-13T14:47:55.111Z</t>
+    <t>2026-10-13T15:20:11.055Z</t>
   </si>
   <si>
     <t>Business Development Leaders | Destination Pet</t>
@@ -502,7 +502,7 @@
     <t>about-us/meet-the-team/leadership</t>
   </si>
   <si>
-    <t>2026-10-13T14:47:59.037Z</t>
+    <t>2026-10-13T15:20:16.502Z</t>
   </si>
   <si>
     <t>Leadership - Meet the team | Destination Pet</t>

</xml_diff>